<commit_message>
Updated 2026 October 22
</commit_message>
<xml_diff>
--- a/4_results/e_QA/Results_vs_ICRP145_electrons.xlsx
+++ b/4_results/e_QA/Results_vs_ICRP145_electrons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04\home\clarence\Geant4_SAF_Calculations\PHITS_Geant4_python_scripts\4_results\e_QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F1D92C-9C50-480C-9577-AE6EB2247A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A146D6-A360-4577-8B05-CC8E6396B0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{727AC7D9-CB15-476D-9018-9B172206195C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{727AC7D9-CB15-476D-9018-9B172206195C}"/>
   </bookViews>
   <sheets>
     <sheet name="Cortical_bone" sheetId="1" r:id="rId1"/>
@@ -1486,104 +1486,128 @@
       <c r="A8" s="1">
         <v>0.01</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9" t="e">
+      <c r="C8" s="8">
+        <v>0.42241819350454801</v>
+      </c>
+      <c r="D8" s="9">
         <f>((B8-C8)/C8)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F8" s="1">
         <v>0.01</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="9" t="e">
-        <f t="shared" ref="I8:I10" si="0">((G8-H8)/H8)*100</f>
-        <v>#DIV/0!</v>
+      <c r="H8" s="8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="9">
+        <f>IFERROR((((G8-H8)/H8)*100), 0)</f>
+        <v>0</v>
       </c>
       <c r="K8" s="1">
         <v>0.01</v>
       </c>
-      <c r="M8" s="8"/>
-      <c r="N8" s="9" t="e">
+      <c r="M8" s="8">
+        <v>1.6716285892174799E-7</v>
+      </c>
+      <c r="N8" s="9">
         <f>((L8-M8)/M8)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>0.1</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9" t="e">
+      <c r="C9" s="8">
+        <v>0.42241819350454801</v>
+      </c>
+      <c r="D9" s="9">
         <f>((B9-C9)/C9)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F9" s="1">
         <v>0.1</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="9" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+      <c r="H9" s="8">
+        <v>1.47307226435298E-5</v>
+      </c>
+      <c r="I9" s="9">
+        <f t="shared" ref="I8:I10" si="0">((G9-H9)/H9)*100</f>
+        <v>-100</v>
       </c>
       <c r="K9" s="1">
         <v>0.1</v>
       </c>
-      <c r="M9" s="8"/>
-      <c r="N9" s="9" t="e">
+      <c r="M9" s="8">
+        <v>8.4259667607641296E-5</v>
+      </c>
+      <c r="N9" s="9">
         <f t="shared" ref="N9:N10" si="1">((L9-M9)/M9)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9" t="e">
+      <c r="C10" s="8">
+        <v>0.40914873439486099</v>
+      </c>
+      <c r="D10" s="9">
         <f>((B10-C10)/C10)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="9" t="e">
+      <c r="H10" s="8">
+        <v>1.2401035352988901E-3</v>
+      </c>
+      <c r="I10" s="9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
       </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="9" t="e">
+      <c r="M10" s="8">
+        <v>3.3800670771468601E-3</v>
+      </c>
+      <c r="N10" s="9">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9" t="e">
+      <c r="C11" s="8">
+        <v>0.30559658326523498</v>
+      </c>
+      <c r="D11" s="9">
         <f>((B11-C11)/C11)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F11" s="1">
         <v>10</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="9" t="e">
+      <c r="H11" s="8">
+        <v>1.0898914150641601E-2</v>
+      </c>
+      <c r="I11" s="9">
         <f>((G11-H11)/H11)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="K11" s="1">
         <v>10</v>
       </c>
-      <c r="M11" s="8"/>
-      <c r="N11" s="9" t="e">
+      <c r="M11" s="8">
+        <v>2.14081263497687E-2</v>
+      </c>
+      <c r="N11" s="9">
         <f>((L11-M11)/M11)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1679,104 +1703,128 @@
       <c r="A16" s="1">
         <v>0.01</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="9" t="e">
+      <c r="C16" s="7">
+        <v>1.6302151350209601E-7</v>
+      </c>
+      <c r="D16" s="9">
         <f>((B16-C16)/C16)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F16" s="1">
         <v>0.01</v>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="7">
+        <v>1.1500822414335301E-5</v>
+      </c>
       <c r="I16" s="9">
         <f>IFERROR((((G16-H16)/H16)*100), 0)</f>
+        <v>-100</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="M16" s="7">
         <v>0</v>
       </c>
-      <c r="K16" s="1">
-        <v>0.01</v>
-      </c>
-      <c r="M16" s="7"/>
-      <c r="N16" s="9" t="e">
-        <f t="shared" ref="N16:N18" si="2">((L16-M16)/M16)*100</f>
-        <v>#DIV/0!</v>
+      <c r="N16" s="9">
+        <f>IFERROR((((L16-M16)/M16)*100), 0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>0.1</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="9" t="e">
+      <c r="C17" s="7">
+        <v>1.21818783714023E-4</v>
+      </c>
+      <c r="D17" s="9">
         <f>((B17-C17)/C17)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F17" s="1">
         <v>0.1</v>
       </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="9" t="e">
-        <f t="shared" ref="I17:I18" si="3">((G17-H17)/H17)*100</f>
-        <v>#DIV/0!</v>
+      <c r="H17" s="7">
+        <v>3.65386860959693E-3</v>
+      </c>
+      <c r="I17" s="9">
+        <f t="shared" ref="I17:I18" si="2">((G17-H17)/H17)*100</f>
+        <v>-100</v>
       </c>
       <c r="K17" s="1">
         <v>0.1</v>
       </c>
-      <c r="M17" s="7"/>
-      <c r="N17" s="9" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+      <c r="M17" s="7">
+        <v>2.4901555284303702E-6</v>
+      </c>
+      <c r="N17" s="9">
+        <f t="shared" ref="N16:N18" si="3">((L17-M17)/M17)*100</f>
+        <v>-100</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>1</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="9" t="e">
+      <c r="C18" s="7">
+        <v>6.4292950761299103E-3</v>
+      </c>
+      <c r="D18" s="9">
         <f>((B18-C18)/C18)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
       </c>
-      <c r="H18" s="7"/>
-      <c r="I18" s="9" t="e">
+      <c r="H18" s="7">
+        <v>8.6950272629167893E-2</v>
+      </c>
+      <c r="I18" s="9">
+        <f t="shared" si="2"/>
+        <v>-100</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="M18" s="7">
+        <v>4.3803571190412298E-5</v>
+      </c>
+      <c r="N18" s="9">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K18" s="1">
-        <v>1</v>
-      </c>
-      <c r="M18" s="7"/>
-      <c r="N18" s="9" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>10</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="9" t="e">
+      <c r="C19" s="7">
+        <v>4.4563538474702701E-2</v>
+      </c>
+      <c r="D19" s="9">
         <f>((B19-C19)/C19)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="F19" s="1">
         <v>10</v>
       </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="9" t="e">
+      <c r="H19" s="7">
+        <v>0.19749064066963301</v>
+      </c>
+      <c r="I19" s="9">
         <f>((G19-H19)/H19)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
       <c r="K19" s="1">
         <v>10</v>
       </c>
-      <c r="M19" s="7"/>
-      <c r="N19" s="9" t="e">
+      <c r="M19" s="7">
+        <v>5.5626656380969603E-3</v>
+      </c>
+      <c r="N19" s="9">
         <f>((L19-M19)/M19)*100</f>
-        <v>#DIV/0!</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated 2026 October 23
</commit_message>
<xml_diff>
--- a/4_results/e_QA/Results_vs_ICRP145_electrons.xlsx
+++ b/4_results/e_QA/Results_vs_ICRP145_electrons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04\home\clarence\Geant4_SAF_Calculations\PHITS_Geant4_python_scripts\4_results\e_QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1F7812-56EE-48CA-A964-F208A70AA815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A980D825-251A-42BE-BF69-B18A5A010AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{727AC7D9-CB15-476D-9018-9B172206195C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{727AC7D9-CB15-476D-9018-9B172206195C}"/>
   </bookViews>
   <sheets>
     <sheet name="Cortical_bone" sheetId="1" r:id="rId1"/>
@@ -1489,15 +1489,21 @@
       <c r="A8" s="1">
         <v>0.01</v>
       </c>
+      <c r="B8">
+        <v>0.42372260891431901</v>
+      </c>
       <c r="C8" s="7">
         <v>0.42241819350454801</v>
       </c>
       <c r="D8" s="9">
         <f>((B8-C8)/C8)*100</f>
-        <v>-100</v>
+        <v>0.30879716589596984</v>
       </c>
       <c r="F8" s="1">
         <v>0.01</v>
+      </c>
+      <c r="G8" s="5">
+        <v>5.5409698591035702E-9</v>
       </c>
       <c r="H8" s="7">
         <v>0</v>
@@ -1509,108 +1515,138 @@
       <c r="K8" s="1">
         <v>0.01</v>
       </c>
+      <c r="L8" s="5">
+        <v>1.9679577032950799E-7</v>
+      </c>
       <c r="M8" s="7">
         <v>1.6716285892174799E-7</v>
       </c>
       <c r="N8" s="9">
         <f>((L8-M8)/M8)*100</f>
-        <v>-100</v>
+        <v>17.726970930565212</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>0.1</v>
       </c>
+      <c r="B9">
+        <v>0.42331692505511898</v>
+      </c>
       <c r="C9" s="7">
         <v>0.42241819350454801</v>
       </c>
       <c r="D9" s="9">
         <f>((B9-C9)/C9)*100</f>
-        <v>-100</v>
+        <v>0.21275872213616845</v>
       </c>
       <c r="F9" s="1">
         <v>0.1</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1.57594152711519E-5</v>
       </c>
       <c r="H9" s="7">
         <v>1.47307226435298E-5</v>
       </c>
       <c r="I9" s="9">
-        <f t="shared" ref="I8:I10" si="0">((G9-H9)/H9)*100</f>
-        <v>-100</v>
+        <f t="shared" ref="I9:I10" si="0">((G9-H9)/H9)*100</f>
+        <v>6.9833140743705115</v>
       </c>
       <c r="K9" s="1">
         <v>0.1</v>
+      </c>
+      <c r="L9" s="5">
+        <v>8.9061667034339594E-5</v>
       </c>
       <c r="M9" s="7">
         <v>8.4259667607641296E-5</v>
       </c>
       <c r="N9" s="9">
         <f t="shared" ref="N9:N10" si="1">((L9-M9)/M9)*100</f>
-        <v>-100</v>
+        <v>5.6990486231906488</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1</v>
       </c>
+      <c r="B10">
+        <v>0.41294050565965301</v>
+      </c>
       <c r="C10" s="7">
         <v>0.40914873439486099</v>
       </c>
       <c r="D10" s="9">
         <f>((B10-C10)/C10)*100</f>
-        <v>-100</v>
+        <v>0.92674642398689677</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1.0608989126953999E-3</v>
       </c>
       <c r="H10" s="7">
         <v>1.2401035352988901E-3</v>
       </c>
       <c r="I10" s="9">
         <f t="shared" si="0"/>
-        <v>-100</v>
+        <v>-14.450779108560333</v>
       </c>
       <c r="K10" s="1">
         <v>1</v>
+      </c>
+      <c r="L10">
+        <v>3.4457576598166E-3</v>
       </c>
       <c r="M10" s="7">
         <v>3.3800670771468601E-3</v>
       </c>
       <c r="N10" s="9">
         <f t="shared" si="1"/>
-        <v>-100</v>
+        <v>1.9434697942500543</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
+      <c r="B11">
+        <v>0.30720564983600301</v>
+      </c>
       <c r="C11" s="7">
         <v>0.30559658326523498</v>
       </c>
       <c r="D11" s="9">
         <f>((B11-C11)/C11)*100</f>
-        <v>-100</v>
+        <v>0.52653290608667791</v>
       </c>
       <c r="F11" s="1">
         <v>10</v>
+      </c>
+      <c r="G11">
+        <v>1.1236656773438901E-2</v>
       </c>
       <c r="H11" s="7">
         <v>1.0898914150641601E-2</v>
       </c>
       <c r="I11" s="9">
         <f>((G11-H11)/H11)*100</f>
-        <v>-100</v>
+        <v>3.0988648789147288</v>
       </c>
       <c r="K11" s="1">
         <v>10</v>
+      </c>
+      <c r="L11">
+        <v>2.1406111759811001E-2</v>
       </c>
       <c r="M11" s="7">
         <v>2.14081263497687E-2</v>
       </c>
       <c r="N11" s="9">
         <f>((L11-M11)/M11)*100</f>
-        <v>-100</v>
+        <v>-9.4103982982173227E-3</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1706,25 +1742,34 @@
       <c r="A16" s="1">
         <v>0.01</v>
       </c>
+      <c r="B16" s="5">
+        <v>1.95535987611188E-7</v>
+      </c>
       <c r="C16" s="7">
         <v>1.6302151350209601E-7</v>
       </c>
       <c r="D16" s="9">
         <f>((B16-C16)/C16)*100</f>
-        <v>-100</v>
+        <v>19.944897707426783</v>
       </c>
       <c r="F16" s="1">
         <v>0.01</v>
+      </c>
+      <c r="G16" s="5">
+        <v>1.13451111658149E-5</v>
       </c>
       <c r="H16" s="7">
         <v>1.1500822414335301E-5</v>
       </c>
       <c r="I16" s="9">
         <f>IFERROR((((G16-H16)/H16)*100), 0)</f>
-        <v>-100</v>
+        <v>-1.3539140324983499</v>
       </c>
       <c r="K16" s="1">
         <v>0.01</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
       </c>
       <c r="M16" s="7">
         <v>0</v>
@@ -1738,96 +1783,123 @@
       <c r="A17" s="1">
         <v>0.1</v>
       </c>
+      <c r="B17">
+        <v>1.2518301803299999E-4</v>
+      </c>
       <c r="C17" s="7">
         <v>1.21818783714023E-4</v>
       </c>
       <c r="D17" s="9">
         <f>((B17-C17)/C17)*100</f>
-        <v>-100</v>
+        <v>2.7616712434715569</v>
       </c>
       <c r="F17" s="1">
         <v>0.1</v>
+      </c>
+      <c r="G17">
+        <v>3.6272154958916E-3</v>
       </c>
       <c r="H17" s="7">
         <v>3.65386860959693E-3</v>
       </c>
       <c r="I17" s="9">
         <f t="shared" ref="I17:I18" si="2">((G17-H17)/H17)*100</f>
-        <v>-100</v>
+        <v>-0.72944915521388287</v>
       </c>
       <c r="K17" s="1">
         <v>0.1</v>
+      </c>
+      <c r="L17" s="5">
+        <v>2.6073242253567098E-6</v>
       </c>
       <c r="M17" s="7">
         <v>2.4901555284303702E-6</v>
       </c>
       <c r="N17" s="9">
-        <f t="shared" ref="N16:N18" si="3">((L17-M17)/M17)*100</f>
-        <v>-100</v>
+        <f t="shared" ref="N17:N18" si="3">((L17-M17)/M17)*100</f>
+        <v>4.7052762604027016</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>1</v>
       </c>
+      <c r="B18">
+        <v>6.3193059066653998E-3</v>
+      </c>
       <c r="C18" s="7">
         <v>6.4292950761299103E-3</v>
       </c>
       <c r="D18" s="9">
         <f>((B18-C18)/C18)*100</f>
-        <v>-100</v>
+        <v>-1.7107500614315891</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
+      </c>
+      <c r="G18">
+        <v>8.7091549482682495E-2</v>
       </c>
       <c r="H18" s="7">
         <v>8.6950272629167893E-2</v>
       </c>
       <c r="I18" s="9">
         <f t="shared" si="2"/>
-        <v>-100</v>
+        <v>0.16248005813291716</v>
       </c>
       <c r="K18" s="1">
         <v>1</v>
+      </c>
+      <c r="L18" s="5">
+        <v>3.96341595821806E-5</v>
       </c>
       <c r="M18" s="7">
         <v>4.3803571190412298E-5</v>
       </c>
       <c r="N18" s="9">
         <f t="shared" si="3"/>
-        <v>-100</v>
+        <v>-9.5184285091903558</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>10</v>
       </c>
+      <c r="B19">
+        <v>4.4409497780318399E-2</v>
+      </c>
       <c r="C19" s="7">
         <v>4.4563538474702701E-2</v>
       </c>
       <c r="D19" s="9">
         <f>((B19-C19)/C19)*100</f>
-        <v>-100</v>
+        <v>-0.3456653121738642</v>
       </c>
       <c r="F19" s="1">
         <v>10</v>
+      </c>
+      <c r="G19">
+        <v>0.196730967616907</v>
       </c>
       <c r="H19" s="7">
         <v>0.19749064066963301</v>
       </c>
       <c r="I19" s="9">
         <f>((G19-H19)/H19)*100</f>
-        <v>-100</v>
+        <v>-0.38466281245034056</v>
       </c>
       <c r="K19" s="1">
         <v>10</v>
+      </c>
+      <c r="L19">
+        <v>5.6653564139913003E-3</v>
       </c>
       <c r="M19" s="7">
         <v>5.5626656380969603E-3</v>
       </c>
       <c r="N19" s="9">
         <f>((L19-M19)/M19)*100</f>
-        <v>-100</v>
+        <v>1.8460713365736552</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -3589,15 +3661,21 @@
       <c r="A24" s="1">
         <v>0.01</v>
       </c>
+      <c r="B24">
+        <v>51.395261154460897</v>
+      </c>
       <c r="C24" s="7">
         <v>51.119062222008999</v>
       </c>
       <c r="D24" s="9">
         <f>((B24-C24)/C24)*100</f>
-        <v>-100</v>
+        <v>0.54030516297887432</v>
       </c>
       <c r="F24" s="1">
         <v>0.01</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
       </c>
       <c r="H24" s="7">
         <v>0</v>
@@ -3609,6 +3687,9 @@
       <c r="K24" s="1">
         <v>0.01</v>
       </c>
+      <c r="L24" s="5">
+        <v>5.3235800442035301E-7</v>
+      </c>
       <c r="M24" s="3">
         <v>0</v>
       </c>
@@ -3621,96 +3702,123 @@
       <c r="A25" s="1">
         <v>0.1</v>
       </c>
+      <c r="B25">
+        <v>51.127937183488498</v>
+      </c>
       <c r="C25" s="7">
         <v>50.884653851084103</v>
       </c>
       <c r="D25" s="9">
         <f>((B25-C25)/C25)*100</f>
-        <v>-100</v>
+        <v>0.47810747247367252</v>
       </c>
       <c r="F25" s="1">
         <v>0.1</v>
+      </c>
+      <c r="G25" s="5">
+        <v>5.3001905245369397E-6</v>
       </c>
       <c r="H25" s="7">
         <v>4.95990501473595E-6</v>
       </c>
       <c r="I25" s="9">
         <f>((G25-H25)/H25)*100</f>
-        <v>-100</v>
+        <v>6.8607263403229801</v>
       </c>
       <c r="K25" s="1">
         <v>0.1</v>
+      </c>
+      <c r="L25">
+        <v>2.0347190966739999E-4</v>
       </c>
       <c r="M25" s="3">
         <v>1.9909727635756999E-4</v>
       </c>
       <c r="N25" s="9">
-        <f t="shared" ref="N24:N26" si="4">((L25-M25)/M25)*100</f>
-        <v>-100</v>
+        <f t="shared" ref="N25:N26" si="4">((L25-M25)/M25)*100</f>
+        <v>2.1972341309046102</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>1</v>
       </c>
+      <c r="B26">
+        <v>44.1219001200365</v>
+      </c>
       <c r="C26" s="7">
         <v>41.3777117016988</v>
       </c>
       <c r="D26" s="9">
         <f>((B26-C26)/C26)*100</f>
-        <v>-100</v>
+        <v>6.6320448992471341</v>
       </c>
       <c r="F26" s="1">
         <v>1</v>
+      </c>
+      <c r="G26" s="5">
+        <v>4.2760292512648798E-5</v>
       </c>
       <c r="H26" s="7">
         <v>4.3027394250357499E-5</v>
       </c>
       <c r="I26" s="9">
         <f>((G26-H26)/H26)*100</f>
-        <v>-100</v>
+        <v>-0.62077135360452729</v>
       </c>
       <c r="K26" s="1">
         <v>1</v>
+      </c>
+      <c r="L26">
+        <v>0.120310325518747</v>
       </c>
       <c r="M26" s="3">
         <v>0.121370238263066</v>
       </c>
       <c r="N26" s="9">
         <f t="shared" si="4"/>
-        <v>-100</v>
+        <v>-0.87328883875277508</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>10</v>
       </c>
+      <c r="B27">
+        <v>10.3502142947873</v>
+      </c>
       <c r="C27" s="7">
         <v>9.20602074697854</v>
       </c>
       <c r="D27" s="9">
         <f>((B27-C27)/C27)*100</f>
-        <v>-100</v>
+        <v>12.428752652814621</v>
       </c>
       <c r="F27" s="1">
         <v>10</v>
+      </c>
+      <c r="G27">
+        <v>1.64112606793657E-2</v>
       </c>
       <c r="H27" s="7">
         <v>2.2804722106308201E-2</v>
       </c>
       <c r="I27" s="9">
         <f>((G27-H27)/H27)*100</f>
-        <v>-100</v>
+        <v>-28.035691016703744</v>
       </c>
       <c r="K27" s="1">
         <v>10</v>
+      </c>
+      <c r="L27">
+        <v>0.75492018672251204</v>
       </c>
       <c r="M27" s="3">
         <v>0.73987595206097401</v>
       </c>
       <c r="N27" s="9">
         <f>((L27-M27)/M27)*100</f>
-        <v>-100</v>
+        <v>2.033345538482676</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -3806,6 +3914,9 @@
       <c r="A32" s="1">
         <v>0.01</v>
       </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
       <c r="C32" s="3">
         <v>0</v>
       </c>
@@ -3816,6 +3927,9 @@
       <c r="F32" s="1">
         <v>0.01</v>
       </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
       <c r="H32" s="3">
         <v>0</v>
       </c>
@@ -3826,6 +3940,9 @@
       <c r="K32" s="1">
         <v>0.01</v>
       </c>
+      <c r="L32">
+        <v>0</v>
+      </c>
       <c r="M32" s="3">
         <v>0</v>
       </c>
@@ -3838,96 +3955,123 @@
       <c r="A33" s="1">
         <v>0.1</v>
       </c>
+      <c r="B33">
+        <v>1.064474713841E-4</v>
+      </c>
       <c r="C33" s="3">
         <v>1.0494911193046001E-4</v>
       </c>
       <c r="D33" s="9">
-        <f t="shared" ref="D32:D34" si="5">((B33-C33)/C33)*100</f>
-        <v>-100</v>
+        <f t="shared" ref="D33:D34" si="5">((B33-C33)/C33)*100</f>
+        <v>1.4277009362716835</v>
       </c>
       <c r="F33" s="1">
         <v>0.1</v>
+      </c>
+      <c r="G33" s="5">
+        <v>1.8508466629028399E-5</v>
       </c>
       <c r="H33" s="3">
         <v>2.2376626591342801E-5</v>
       </c>
       <c r="I33" s="9">
         <f t="shared" ref="I33:I34" si="6">((G33-H33)/H33)*100</f>
-        <v>-100</v>
+        <v>-17.286609071855978</v>
       </c>
       <c r="K33" s="1">
         <v>0.1</v>
+      </c>
+      <c r="L33" s="5">
+        <v>6.5552707406012196E-6</v>
       </c>
       <c r="M33" s="3">
         <v>6.2142459259582401E-6</v>
       </c>
       <c r="N33" s="9">
-        <f t="shared" ref="N32:N34" si="7">((L33-M33)/M33)*100</f>
-        <v>-100</v>
+        <f t="shared" ref="N33:N34" si="7">((L33-M33)/M33)*100</f>
+        <v>5.4877907747172614</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>1</v>
       </c>
+      <c r="B34">
+        <v>5.5043583609019995E-4</v>
+      </c>
       <c r="C34" s="3">
         <v>5.69173646801353E-4</v>
       </c>
       <c r="D34" s="9">
         <f t="shared" si="5"/>
-        <v>-100</v>
+        <v>-3.29210792109859</v>
       </c>
       <c r="F34" s="1">
         <v>1</v>
+      </c>
+      <c r="G34">
+        <v>1.3389722428999999E-4</v>
       </c>
       <c r="H34" s="3">
         <v>1.7000150190338799E-4</v>
       </c>
       <c r="I34" s="9">
         <f t="shared" si="6"/>
-        <v>-100</v>
+        <v>-21.237622732242738</v>
       </c>
       <c r="K34" s="1">
         <v>1</v>
+      </c>
+      <c r="L34" s="5">
+        <v>5.87291884769156E-5</v>
       </c>
       <c r="M34" s="3">
         <v>5.7587817224647203E-5</v>
       </c>
       <c r="N34" s="9">
         <f t="shared" si="7"/>
-        <v>-100</v>
+        <v>1.9819665117987797</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>10</v>
       </c>
+      <c r="B35">
+        <v>0.56488598166639803</v>
+      </c>
       <c r="C35" s="3">
         <v>0.56917360310003595</v>
       </c>
       <c r="D35" s="9">
         <f>((B35-C35)/C35)*100</f>
-        <v>-100</v>
+        <v>-0.75330644469194497</v>
       </c>
       <c r="F35" s="1">
         <v>10</v>
+      </c>
+      <c r="G35">
+        <v>0.100480348859501</v>
       </c>
       <c r="H35" s="3">
         <v>0.134144239027183</v>
       </c>
       <c r="I35" s="9">
         <f>((G35-H35)/H35)*100</f>
-        <v>-100</v>
+        <v>-25.095293254345684</v>
       </c>
       <c r="K35" s="1">
         <v>10</v>
+      </c>
+      <c r="L35">
+        <v>1.2660511946139499E-2</v>
       </c>
       <c r="M35" s="3">
         <v>1.3052762747487699E-2</v>
       </c>
       <c r="N35" s="9">
         <f>((L35-M35)/M35)*100</f>
-        <v>-100</v>
+        <v>-3.0051170693629397</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>